<commit_message>
[ADD] No multicollinearity results
</commit_message>
<xml_diff>
--- a/results/metrics_modelling2.xlsx
+++ b/results/metrics_modelling2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,19 +487,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.8266666666666667</v>
+        <v>0.8</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8686868686868686</v>
+        <v>0.845360824742268</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.8367346938775511</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8958333333333334</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="H2" t="n">
-        <v>0.7997685185185186</v>
+        <v>0.7789351851851851</v>
       </c>
     </row>
     <row r="3">
@@ -519,19 +519,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.8</v>
+        <v>0.8133333333333334</v>
       </c>
       <c r="E3" t="n">
         <v>0.8571428571428572</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.84</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9375</v>
+        <v>0.875</v>
       </c>
       <c r="H3" t="n">
-        <v>0.7465277777777777</v>
+        <v>0.7893518518518519</v>
       </c>
     </row>
     <row r="4">
@@ -551,19 +551,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.8266666666666667</v>
+        <v>0.8</v>
       </c>
       <c r="E4" t="n">
-        <v>0.8686868686868686</v>
+        <v>0.845360824742268</v>
       </c>
       <c r="F4" t="n">
-        <v>0.8431372549019608</v>
+        <v>0.8367346938775511</v>
       </c>
       <c r="G4" t="n">
-        <v>0.8958333333333334</v>
+        <v>0.8541666666666666</v>
       </c>
       <c r="H4" t="n">
-        <v>0.7997685185185186</v>
+        <v>0.7789351851851851</v>
       </c>
     </row>
     <row r="5">
@@ -586,16 +586,16 @@
         <v>0.8</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8571428571428572</v>
+        <v>0.854368932038835</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7894736842105263</v>
+        <v>0.8</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9375</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="H5" t="n">
-        <v>0.7465277777777777</v>
+        <v>0.7546296296296295</v>
       </c>
     </row>
     <row r="6">
@@ -615,19 +615,19 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.6266666666666667</v>
+        <v>0.8266666666666667</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8659793814432989</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.875</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6435185185185186</v>
+        <v>0.8078703703703703</v>
       </c>
     </row>
     <row r="7">
@@ -647,19 +647,19 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.7733333333333333</v>
+        <v>0.7866666666666666</v>
       </c>
       <c r="E7" t="n">
-        <v>0.8440366972477064</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="F7" t="n">
-        <v>0.7540983606557377</v>
+        <v>0.7857142857142857</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9583333333333334</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="H7" t="n">
-        <v>0.7013888888888888</v>
+        <v>0.7361111111111112</v>
       </c>
     </row>
     <row r="8">
@@ -679,19 +679,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.6266666666666667</v>
+        <v>0.84</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8695652173913043</v>
       </c>
       <c r="F8" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6435185185185186</v>
+        <v>0.8425925925925926</v>
       </c>
     </row>
     <row r="9">
@@ -714,16 +714,16 @@
         <v>0.7733333333333333</v>
       </c>
       <c r="E9" t="n">
-        <v>0.8440366972477064</v>
+        <v>0.8349514563106797</v>
       </c>
       <c r="F9" t="n">
-        <v>0.7540983606557377</v>
+        <v>0.7818181818181819</v>
       </c>
       <c r="G9" t="n">
-        <v>0.9583333333333334</v>
+        <v>0.8958333333333334</v>
       </c>
       <c r="H9" t="n">
-        <v>0.7013888888888888</v>
+        <v>0.7256944444444445</v>
       </c>
     </row>
     <row r="10">
@@ -743,19 +743,19 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.7733333333333333</v>
+        <v>0.8</v>
       </c>
       <c r="E10" t="n">
-        <v>0.8282828282828283</v>
+        <v>0.8421052631578947</v>
       </c>
       <c r="F10" t="n">
-        <v>0.803921568627451</v>
+        <v>0.851063829787234</v>
       </c>
       <c r="G10" t="n">
-        <v>0.8541666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="H10" t="n">
-        <v>0.7418981481481481</v>
+        <v>0.7870370370370371</v>
       </c>
     </row>
     <row r="11">
@@ -775,19 +775,19 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.7733333333333333</v>
+        <v>0.8266666666666667</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8349514563106797</v>
+        <v>0.8659793814432989</v>
       </c>
       <c r="F11" t="n">
-        <v>0.7818181818181819</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="G11" t="n">
-        <v>0.8958333333333334</v>
+        <v>0.875</v>
       </c>
       <c r="H11" t="n">
-        <v>0.7256944444444445</v>
+        <v>0.8078703703703703</v>
       </c>
     </row>
     <row r="12">
@@ -807,19 +807,19 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.7733333333333333</v>
+        <v>0.8266666666666667</v>
       </c>
       <c r="E12" t="n">
-        <v>0.8282828282828283</v>
+        <v>0.8602150537634408</v>
       </c>
       <c r="F12" t="n">
-        <v>0.803921568627451</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="G12" t="n">
-        <v>0.8541666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="H12" t="n">
-        <v>0.7418981481481481</v>
+        <v>0.8240740740740742</v>
       </c>
     </row>
     <row r="13">
@@ -839,19 +839,19 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.7733333333333333</v>
+        <v>0.8266666666666667</v>
       </c>
       <c r="E13" t="n">
-        <v>0.8349514563106797</v>
+        <v>0.8686868686868686</v>
       </c>
       <c r="F13" t="n">
-        <v>0.7818181818181819</v>
+        <v>0.8431372549019608</v>
       </c>
       <c r="G13" t="n">
         <v>0.8958333333333334</v>
       </c>
       <c r="H13" t="n">
-        <v>0.7256944444444445</v>
+        <v>0.7997685185185186</v>
       </c>
     </row>
     <row r="14">
@@ -999,19 +999,19 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.8</v>
+        <v>0.8533333333333334</v>
       </c>
       <c r="E18" t="n">
-        <v>0.6938775510204082</v>
+        <v>0.7659574468085106</v>
       </c>
       <c r="F18" t="n">
-        <v>0.5862068965517241</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G18" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="H18" t="n">
-        <v>0.8159090909090909</v>
+        <v>0.8681818181818182</v>
       </c>
     </row>
     <row r="19">
@@ -1031,19 +1031,19 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.88</v>
       </c>
       <c r="E19" t="n">
-        <v>0.7368421052631577</v>
+        <v>0.7804878048780488</v>
       </c>
       <c r="F19" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.7619047619047619</v>
       </c>
       <c r="G19" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="H19" t="n">
-        <v>0.8136363636363635</v>
+        <v>0.8545454545454545</v>
       </c>
     </row>
     <row r="20">
@@ -1063,19 +1063,19 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.8</v>
+        <v>0.8266666666666667</v>
       </c>
       <c r="E20" t="n">
-        <v>0.6938775510204082</v>
+        <v>0.723404255319149</v>
       </c>
       <c r="F20" t="n">
-        <v>0.5862068965517241</v>
+        <v>0.6296296296296297</v>
       </c>
       <c r="G20" t="n">
         <v>0.85</v>
       </c>
       <c r="H20" t="n">
-        <v>0.8159090909090909</v>
+        <v>0.8340909090909091</v>
       </c>
     </row>
     <row r="21">
@@ -1095,19 +1095,19 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.8933333333333333</v>
       </c>
       <c r="E21" t="n">
-        <v>0.7368421052631577</v>
+        <v>0.8000000000000002</v>
       </c>
       <c r="F21" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.8</v>
       </c>
       <c r="G21" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="H21" t="n">
-        <v>0.8136363636363635</v>
+        <v>0.8636363636363636</v>
       </c>
     </row>
     <row r="22">
@@ -1127,19 +1127,19 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.4933333333333333</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="E22" t="n">
-        <v>0.4864864864864865</v>
+        <v>0.7826086956521738</v>
       </c>
       <c r="F22" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.6923076923076923</v>
       </c>
       <c r="G22" t="n">
         <v>0.9</v>
       </c>
       <c r="H22" t="n">
-        <v>0.6227272727272728</v>
+        <v>0.8772727272727272</v>
       </c>
     </row>
     <row r="23">
@@ -1159,19 +1159,19 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>0.7368421052631577</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="H23" t="n">
-        <v>0.5</v>
+        <v>0.8136363636363635</v>
       </c>
     </row>
     <row r="24">
@@ -1191,19 +1191,19 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.4933333333333333</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="E24" t="n">
-        <v>0.4864864864864865</v>
+        <v>0.7826086956521738</v>
       </c>
       <c r="F24" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.6923076923076923</v>
       </c>
       <c r="G24" t="n">
         <v>0.9</v>
       </c>
       <c r="H24" t="n">
-        <v>0.6227272727272728</v>
+        <v>0.8772727272727272</v>
       </c>
     </row>
     <row r="25">
@@ -1223,19 +1223,19 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.9066666666666666</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>0.8205128205128205</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>0.8421052631578947</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="H25" t="n">
-        <v>0.5</v>
+        <v>0.8727272727272728</v>
       </c>
     </row>
     <row r="26">
@@ -1255,19 +1255,19 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.8533333333333334</v>
       </c>
       <c r="E26" t="n">
-        <v>0.6153846153846154</v>
+        <v>0.7555555555555556</v>
       </c>
       <c r="F26" t="n">
-        <v>0.5</v>
+        <v>0.68</v>
       </c>
       <c r="G26" t="n">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="H26" t="n">
-        <v>0.7545454545454545</v>
+        <v>0.8522727272727272</v>
       </c>
     </row>
     <row r="27">
@@ -1287,19 +1287,19 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.7733333333333333</v>
+        <v>0.9066666666666666</v>
       </c>
       <c r="E27" t="n">
-        <v>0.5641025641025641</v>
+        <v>0.8292682926829269</v>
       </c>
       <c r="F27" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.8095238095238095</v>
       </c>
       <c r="G27" t="n">
-        <v>0.55</v>
+        <v>0.85</v>
       </c>
       <c r="H27" t="n">
-        <v>0.7022727272727273</v>
+        <v>0.8886363636363637</v>
       </c>
     </row>
     <row r="28">
@@ -1319,19 +1319,19 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.7333333333333333</v>
+        <v>0.8933333333333333</v>
       </c>
       <c r="E28" t="n">
-        <v>0.6153846153846154</v>
+        <v>0.8260869565217392</v>
       </c>
       <c r="F28" t="n">
-        <v>0.5</v>
+        <v>0.7307692307692307</v>
       </c>
       <c r="G28" t="n">
-        <v>0.8</v>
+        <v>0.95</v>
       </c>
       <c r="H28" t="n">
-        <v>0.7545454545454545</v>
+        <v>0.9113636363636364</v>
       </c>
     </row>
     <row r="29">
@@ -1351,19 +1351,19 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.7733333333333333</v>
+        <v>0.88</v>
       </c>
       <c r="E29" t="n">
-        <v>0.5641025641025641</v>
+        <v>0.7906976744186046</v>
       </c>
       <c r="F29" t="n">
-        <v>0.5789473684210527</v>
+        <v>0.7391304347826086</v>
       </c>
       <c r="G29" t="n">
-        <v>0.55</v>
+        <v>0.85</v>
       </c>
       <c r="H29" t="n">
-        <v>0.7022727272727273</v>
+        <v>0.8704545454545455</v>
       </c>
     </row>
     <row r="30">
@@ -1492,6 +1492,1030 @@
       </c>
       <c r="H33" t="n">
         <v>0.9318181818181818</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>logisticregression_smote_splashing_onehot</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.845360824742268</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.8367346938775511</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.8541666666666666</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.7789351851851851</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>logisticregression_splashing_onehot</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0.8266666666666667</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.8686868686868686</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.8431372549019608</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.7997685185185186</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>logisticregression_smote_splashing_ordenc</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>0.7733333333333333</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.8282828282828283</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.803921568627451</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.8541666666666666</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.7418981481481481</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>logisticregression_splashing_ordenc</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.854368932038835</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.7546296296296295</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>svc_smote_splashing_onehot</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.8387096774193549</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.795138888888889</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>svc_splashing_onehot</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>0.7866666666666666</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.7361111111111112</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>svc_smote_splashing_ordenc</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0.8266666666666667</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.8602150537634408</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.8240740740740742</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>svc_splashing_ordenc</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>0.7866666666666666</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.8431372549019608</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.7962962962962963</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.744212962962963</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_smote_splashing_onehot</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.8421052631578947</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.851063829787234</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.7870370370370371</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_splashing_onehot</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>0.7866666666666666</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.7685185185185186</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_smote_splashing_ordenc</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>0.8133333333333334</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.851063829787234</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.8695652173913043</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.8055555555555556</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_splashing_ordenc</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.845360824742268</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.8367346938775511</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.8541666666666666</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.7789351851851851</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>xgbclassifier_smote_splashing</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.8775510204081632</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.8182870370370371</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>xgbclassifier_splashing</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.8865979381443299</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.8775510204081632</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.8368055555555556</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>catboostclassifier_smote_splashing</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.8865979381443299</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.8775510204081632</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.8368055555555556</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>catboostclassifier_splashing</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.8653846153846154</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.8391203703703703</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>logisticregression_smote_net_impact_onehot</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.7659574468085106</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0.8681818181818182</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>logisticregression_net_impact_onehot</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.7804878048780488</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.7619047619047619</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0.8545454545454545</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>logisticregression_smote_net_impact_ordenc</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.7391304347826088</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.6538461538461539</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0.8431818181818183</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>logisticregression_net_impact_ordenc</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>0.8933333333333333</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0.8000000000000002</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0.8636363636363636</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>svc_smote_net_impact_onehot</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>0.8933333333333333</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.8260869565217392</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.7307692307692307</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0.9113636363636364</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>svc_net_impact_onehot</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.7428571428571429</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0.8068181818181818</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>svc_smote_net_impact_ordenc</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0.7826086956521738</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.6923076923076923</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0.8772727272727272</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>svc_net_impact_ordenc</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>0.8933333333333333</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0.7894736842105262</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0.8477272727272728</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_smote_net_impact_onehot</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0.7659574468085106</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0.8681818181818182</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_net_impact_onehot</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0.8571428571428572</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0.9136363636363636</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_smote_net_impact_ordenc</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0.8863636363636364</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_net_impact_ordenc</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0.8780487804878048</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.9227272727272726</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>xgbclassifier_smote_net_impact</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.8717948717948718</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.8947368421052632</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0.9068181818181819</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>xgbclassifier_net_impact</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>0.8933333333333333</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0.7777777777777777</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0.8318181818181818</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>catboostclassifier_smote_net_impact</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0.8780487804878048</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0.9227272727272726</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>df_modelling_no_multicollinearity</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>catboostclassifier_net_impact</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0.8780487804878048</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0.9227272727272726</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[ADD] DF dimensionless results
</commit_message>
<xml_diff>
--- a/results/metrics_modelling2.xlsx
+++ b/results/metrics_modelling2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2518,6 +2518,1030 @@
         <v>0.9227272727272726</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>logisticregression_smote_splashing_onehot</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>0.7866666666666666</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0.7685185185185186</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>logisticregression_splashing_onehot</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0.8799999999999999</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0.8101851851851851</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>logisticregression_smote_splashing_ordenc</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>0.7733333333333333</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0.8282828282828283</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.803921568627451</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0.8541666666666666</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0.7418981481481481</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>logisticregression_splashing_ordenc</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>0.8133333333333334</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0.8653846153846154</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0.8035714285714286</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0.7650462962962963</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>svc_smote_splashing_onehot</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0.888888888888889</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.8627450980392157</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0.8287037037037036</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>svc_splashing_onehot</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0.8571428571428572</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0.7894736842105263</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0.7465277777777777</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>svc_smote_splashing_ordenc</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0.8775510204081632</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H72" t="n">
+        <v>0.8182870370370371</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>svc_splashing_ordenc</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E73" t="n">
+        <v>0.8571428571428572</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0.7894736842105263</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="H73" t="n">
+        <v>0.7465277777777777</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_smote_splashing_onehot</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0.8775510204081632</v>
+      </c>
+      <c r="F74" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H74" t="n">
+        <v>0.8182870370370371</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_splashing_onehot</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0.8910891089108911</v>
+      </c>
+      <c r="F75" t="n">
+        <v>0.8490566037735849</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="H75" t="n">
+        <v>0.8206018518518519</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_smote_splashing_ordenc</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="E76" t="n">
+        <v>0.8979591836734694</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G76" t="n">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="H76" t="n">
+        <v>0.8472222222222222</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_splashing_ordenc</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="E77" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0.8653846153846154</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0.8391203703703703</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>xgbclassifier_smote_splashing</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0.8775510204081632</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0.8182870370370371</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>xgbclassifier_splashing</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E79" t="n">
+        <v>0.8775510204081632</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H79" t="n">
+        <v>0.8182870370370371</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>catboostclassifier_smote_splashing</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="E80" t="n">
+        <v>0.8865979381443299</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0.8775510204081632</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0.8958333333333334</v>
+      </c>
+      <c r="H80" t="n">
+        <v>0.8368055555555556</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>catboostclassifier_splashing</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="E81" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0.8653846153846154</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0.8391203703703703</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>logisticregression_smote_net_impact_onehot</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="E82" t="n">
+        <v>0.7659574468085106</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H82" t="n">
+        <v>0.8681818181818182</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>logisticregression_net_impact_onehot</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0.7692307692307692</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0.7894736842105263</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0.8386363636363635</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>logisticregression_smote_net_impact_ordenc</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="E84" t="n">
+        <v>0.7555555555555556</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0.8522727272727272</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>logisticregression_net_impact_ordenc</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>0.8933333333333333</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0.8000000000000002</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0.8636363636363636</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>svc_smote_net_impact_onehot</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E86" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H86" t="n">
+        <v>0.8863636363636364</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>svc_net_impact_onehot</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="E87" t="n">
+        <v>0.7222222222222223</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0.7977272727272726</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>svc_smote_net_impact_ordenc</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E88" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H88" t="n">
+        <v>0.8863636363636364</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>svc_net_impact_ordenc</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>0.8533333333333334</v>
+      </c>
+      <c r="E89" t="n">
+        <v>0.7027027027027027</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0.7647058823529411</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0.7886363636363636</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_smote_net_impact_onehot</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E90" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H90" t="n">
+        <v>0.859090909090909</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_net_impact_onehot</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E91" t="n">
+        <v>0.7906976744186046</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0.7391304347826086</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0.8704545454545455</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_smote_net_impact_ordenc</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="E92" t="n">
+        <v>0.7826086956521738</v>
+      </c>
+      <c r="F92" t="n">
+        <v>0.6923076923076923</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H92" t="n">
+        <v>0.8772727272727272</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>kneighborsclassifier_net_impact_ordenc</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E93" t="n">
+        <v>0.7906976744186046</v>
+      </c>
+      <c r="F93" t="n">
+        <v>0.7391304347826086</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0.8704545454545455</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>xgbclassifier_smote_net_impact</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E94" t="n">
+        <v>0.8421052631578948</v>
+      </c>
+      <c r="F94" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0.8818181818181818</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>xgbclassifier_net_impact</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>0.8933333333333333</v>
+      </c>
+      <c r="E95" t="n">
+        <v>0.7777777777777777</v>
+      </c>
+      <c r="F95" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H95" t="n">
+        <v>0.8318181818181818</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>catboostclassifier_smote_net_impact</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="E96" t="n">
+        <v>0.8780487804878048</v>
+      </c>
+      <c r="F96" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H96" t="n">
+        <v>0.9227272727272726</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>df_modelling_dimensionless</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>net_impact</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>catboostclassifier_net_impact</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>0.9466666666666667</v>
+      </c>
+      <c r="E97" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F97" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0.9318181818181818</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>